<commit_message>
added reading actionpoints and virtualinstruments from excel
</commit_message>
<xml_diff>
--- a/Source/Tests/resources/test_virtual_config.xlsx
+++ b/Source/Tests/resources/test_virtual_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\HAL\Source\Tests\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{554D32BA-3085-4E43-B091-E7503D167F7E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D1FDB3-3459-40E2-8AF5-B4EF21DA4DDB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" tabRatio="791" xr2:uid="{694A1011-F733-4B3D-865A-EAFA5EFA9CF7}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" tabRatio="791" activeTab="6" xr2:uid="{694A1011-F733-4B3D-865A-EAFA5EFA9CF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Study" sheetId="3" r:id="rId1"/>
@@ -27,11 +27,16 @@
     <sheet name="cDAQ9191-TC9210.ai0" sheetId="7" r:id="rId12"/>
   </sheets>
   <definedNames>
+    <definedName name="ActionPoints" localSheetId="0">Study!$C$2:$C$21</definedName>
     <definedName name="Attributes.Baudrate" localSheetId="8">'CAN1'!$B$5</definedName>
     <definedName name="Attributes.Baudrate" localSheetId="9">'PCAN_USBBUS1  0x51'!$B$5</definedName>
     <definedName name="Attributes.Channels" localSheetId="10">'cDAQ9191-TC9210'!$B$6:$B$14</definedName>
     <definedName name="Attributes.DbcFilepath" localSheetId="8">'CAN1'!$B$7</definedName>
     <definedName name="Attributes.DbcFilepath" localSheetId="9">'PCAN_USBBUS1  0x51'!$B$7</definedName>
+    <definedName name="Attributes.FrameName1" localSheetId="6">'Virtual NEO480 1'!$B$5</definedName>
+    <definedName name="Attributes.FrameName1" localSheetId="7">'Virtual Thermometer'!$B$5</definedName>
+    <definedName name="Attributes.FrameName2" localSheetId="6">'Virtual NEO480 1'!$B$6</definedName>
+    <definedName name="Attributes.FrameName2" localSheetId="7">'Virtual Thermometer'!$B$6</definedName>
     <definedName name="Attributes.GrpcServerAddress" localSheetId="8">'CAN1'!$B$9</definedName>
     <definedName name="Attributes.ReadRate" localSheetId="8">'CAN1'!$B$6</definedName>
     <definedName name="Attributes.ReadRate" localSheetId="10">'cDAQ9191-TC9210'!$B$5</definedName>
@@ -50,10 +55,16 @@
     <definedName name="Class" localSheetId="8">'CAN1'!$B$2</definedName>
     <definedName name="Class" localSheetId="10">'cDAQ9191-TC9210'!$B$2</definedName>
     <definedName name="Class" localSheetId="9">'PCAN_USBBUS1  0x51'!$B$2</definedName>
+    <definedName name="Class" localSheetId="6">'Virtual NEO480 1'!$B$2</definedName>
+    <definedName name="Class" localSheetId="7">'Virtual Thermometer'!$B$2</definedName>
     <definedName name="ConfigureClass" localSheetId="8">'CAN1'!$B$3</definedName>
     <definedName name="ConfigureClass" localSheetId="10">'cDAQ9191-TC9210'!$B$3</definedName>
     <definedName name="ConfigureClass" localSheetId="9">'PCAN_USBBUS1  0x51'!$B$3</definedName>
     <definedName name="Enabled" localSheetId="11">'cDAQ9191-TC9210.ai0'!$B$2</definedName>
+    <definedName name="Identifier" localSheetId="6">'Virtual NEO480 1'!$B$1</definedName>
+    <definedName name="Identifier" localSheetId="7">'Virtual Thermometer'!$B$1</definedName>
+    <definedName name="Instrument" localSheetId="6">'Virtual NEO480 1'!$B$3</definedName>
+    <definedName name="Instrument" localSheetId="7">'Virtual Thermometer'!$B$3</definedName>
     <definedName name="InstrumentIdentifier" localSheetId="8">'CAN1'!$B$1</definedName>
     <definedName name="InstrumentIdentifier" localSheetId="10">'cDAQ9191-TC9210'!$B$1</definedName>
     <definedName name="InstrumentIdentifier" localSheetId="9">'PCAN_USBBUS1  0x51'!$B$1</definedName>
@@ -63,6 +74,7 @@
     <definedName name="Name" localSheetId="11">'cDAQ9191-TC9210.ai0'!$B$1</definedName>
     <definedName name="ThermocoupleType" localSheetId="11">'cDAQ9191-TC9210.ai0'!$B$5</definedName>
     <definedName name="Units" localSheetId="11">'cDAQ9191-TC9210.ai0'!$B$6</definedName>
+    <definedName name="VirtualInstruments" localSheetId="0">Study!$B$2:$B$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -74,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="76">
   <si>
     <t>InstrumentIdentifier</t>
   </si>
@@ -241,15 +253,9 @@
     <t>NEO480A_Msg_1</t>
   </si>
   <si>
-    <t>DataLoggerClass</t>
-  </si>
-  <si>
     <t>SimpleCsvDataLogger.lvclass</t>
   </si>
   <si>
-    <t>DataLogDestination</t>
-  </si>
-  <si>
     <t>D:\hal-logs</t>
   </si>
   <si>
@@ -296,6 +302,18 @@
   </si>
   <si>
     <t>VirtualInstrument</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>Virtual_NEO480_1</t>
+  </si>
+  <si>
+    <t>TC-1</t>
+  </si>
+  <si>
+    <t>Virtual Thermometer.lvclass</t>
   </si>
 </sst>
 </file>
@@ -388,10 +406,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -400,7 +417,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -416,7 +433,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -712,173 +729,144 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBC1553D-31A9-47F1-9003-2533A43CD3A4}">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
     <col min="4" max="4" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="7" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="7" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="4"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="4"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="4"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="4"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="4"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="4"/>
-    </row>
-    <row r="21" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="5"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="6"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="6"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="6"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="6"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="6"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="6"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="6"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="6"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="6"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="6"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="6"/>
+    </row>
+    <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -888,7 +876,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A9D403-72C5-472F-AC2B-4CAB762784A6}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.140625" customWidth="1"/>
     <col min="2" max="2" width="72.42578125" customWidth="1"/>
@@ -951,7 +939,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1380816-54EF-4026-83D9-8EB7D75D6731}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.140625" customWidth="1"/>
     <col min="2" max="2" width="50.85546875" customWidth="1"/>
@@ -1062,7 +1050,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77D67891-1560-40D4-8A09-0C4C9BA29850}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" customWidth="1"/>
@@ -1144,8 +1132,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F12D661-3DBC-4ACA-B17D-ECA2E2886AFC}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
@@ -1153,41 +1141,41 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1197,8 +1185,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B71A4A-0F0A-44DB-B525-8215CC86B044}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
@@ -1206,49 +1194,41 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1258,8 +1238,8 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09D25C40-8A50-421D-9AB2-EF8CA695243E}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
@@ -1267,49 +1247,41 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1319,8 +1291,8 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51A81152-973E-4DD3-BBA3-00065132513E}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
@@ -1328,49 +1300,41 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1380,8 +1344,8 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A3EC77-AECF-4D53-8D81-FDFED6A43D2E}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
@@ -1389,49 +1353,41 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>58</v>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1441,8 +1397,62 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{758A37E4-006D-4EC7-A650-6E18768E6BAD}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{700149C1-66F5-4A24-928F-5BBEDD6006E3}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
@@ -1450,111 +1460,41 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>51</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>52</v>
       </c>
-      <c r="B8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{700149C1-66F5-4A24-928F-5BBEDD6006E3}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="B6" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1566,7 +1506,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A7DE5E1-2065-4857-A2CD-738C548B16E2}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.28515625" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>

</xml_diff>